<commit_message>
fix(excel): calibration impression A4 1-page pour Proforma Anper, GIZ et Tableau Comparatif
Co-authored-by: NigerCertify-offensive-lab <openaiabou@gmail.com>
</commit_message>
<xml_diff>
--- a/proformas-concurrentes/Pro_forma_GIZ.xlsx
+++ b/proformas-concurrentes/Pro_forma_GIZ.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Facture Proforma B" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Facture Proforma B'!$A$1:$E$31</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -29,47 +31,53 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00006633"/>
-      <sz val="13"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
       <i val="1"/>
       <color rgb="00404040"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00505050"/>
+      <sz val="7.8"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00006633"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
       <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00505050"/>
+      <color rgb="00000000"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="8.5"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00006633"/>
-      <sz val="15"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
       <sz val="9.5"/>
     </font>
     <font>
       <name val="Arial"/>
-      <color rgb="00000000"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
+      <i val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00006633"/>
-      <sz val="10.5"/>
+      <sz val="7.5"/>
     </font>
   </fonts>
   <fills count="6">
@@ -81,8 +89,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F0F4F1"/>
-        <bgColor rgb="00F0F4F1"/>
+        <fgColor rgb="00F0F6F2"/>
+        <bgColor rgb="00F0F6F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -114,20 +122,26 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="00B2D8C0"/>
       </left>
       <right style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="00B2D8C0"/>
       </right>
       <top style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="00B2D8C0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00C0C0C0"/>
+        <color rgb="00B2D8C0"/>
       </bottom>
     </border>
     <border>
-      <top style="thin">
+      <left style="thin">
+        <color rgb="00B2D8C0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B2D8C0"/>
+      </right>
+      <top style="medium">
         <color rgb="00006633"/>
       </top>
       <bottom style="double">
@@ -138,25 +152,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -190,6 +203,19 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -554,19 +580,19 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="54" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SAHEL GRAPHIQUE &amp; SÉCURITÉ INDUSTRIELLE (SGSI SA)</t>
@@ -574,11 +600,11 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
-          <t>PROFORMA INVOICE</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
+          <t>PROFORMA INVOICE B</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Solutions d'Étiquetage Technique, Marquage Métrologique &amp; Systèmes de Sécurité</t>
@@ -589,414 +615,426 @@
           <t>Référence N° :</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>SGSI/2026/PF-091</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>Zone Industrielle Yantala, Rue ZI-14, BP 12 850 Niamey — Niger | Tél: (+227) 20 75 18 90 / 90 22 34 56</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
+    <row r="3" ht="13" customHeight="1">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Zone Industrielle Yantala, Rue ZI-14, BP 12 850 Niamey (Niger) | Tél: (+227) 20 75 18 90 / 90 22 34 56</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Date d'émission :</t>
         </is>
       </c>
-      <c r="E3" s="8" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>16/09/2026</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+    <row r="4" ht="13" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>NIF: 52189/S | RCCM: NI-NIA-2019-B-0895 | Email: commercial@sahel-graphique.ne</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Délai de validité :</t>
         </is>
       </c>
-      <c r="E4" s="8" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>90 jours</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>ORGANISME DESTINATAIRE : AGENCE NATIONALE DE LA MÉTROLOGIE ET DE LA CONFORMITÉ (ANMC)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+    <row r="5" ht="6" customHeight="1"/>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>DESTINATAIRE : AGENCE NATIONALE DE LA MÉTROLOGIE ET DE LA CONFORMITÉ (ANMC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Direction Générale — BP 10 700 Niamey (Niger)</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>Identifiant Fiscal NIF : 82397/P</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
-        <is>
-          <t>Objet : Offre de prix pour étiquettes de métrologie et scellés de sécurité personnalisés (campagnes 2027/2028)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="11" t="inlineStr">
+          <t>Direction Générale — BP 10 700 Niamey (République du Niger)</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>NIF Client : 82397/P</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Objet : Offre pour étiquettes de métrologie et scellés de sécurité personnalisés (2027/2028)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="6" customHeight="1"/>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="10" t="inlineStr">
         <is>
           <t>Description détaillée de la prestation / fourniture</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>Quantité</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
-        <is>
-          <t>Prix Unitaire HT (FCFA)</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="inlineStr">
-        <is>
-          <t>Montant Total HT (FCFA)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="12" t="n">
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>P.U. HT (FCFA)</t>
+        </is>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>Total HT (FCFA)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette verte 9cm X 9cm (année 2027, n°6001 à 11000)</t>
         </is>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="13" t="n">
         <v>5000</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="13">
         <f>C11*D11</f>
         <v/>
       </c>
     </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="15" t="n">
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette verte 9cm X 9cm (année 2028, n°0001 à 8000)</t>
         </is>
       </c>
-      <c r="C12" s="17" t="n">
+      <c r="C12" s="16" t="n">
         <v>8000</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="16" t="n">
         <v>200</v>
       </c>
-      <c r="E12" s="17">
+      <c r="E12" s="16">
         <f>C12*D12</f>
         <v/>
       </c>
     </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="12" t="n">
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette orange 9cm X 9cm (n°2001 à 4000)</t>
         </is>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="D13" s="14" t="n">
+      <c r="D13" s="13" t="n">
         <v>200</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="13">
         <f>C13*D13</f>
         <v/>
       </c>
     </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="15" t="n">
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette rouge 9cm X 9cm (n°3001 à 4000)</t>
         </is>
       </c>
-      <c r="C14" s="17" t="n">
+      <c r="C14" s="16" t="n">
         <v>1000</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="16" t="n">
         <v>200</v>
       </c>
-      <c r="E14" s="17">
+      <c r="E14" s="16">
         <f>C14*D14</f>
         <v/>
       </c>
     </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="12" t="n">
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette verte 5,5cm X 5,5cm (année 2027, n°2501 à 3000)</t>
         </is>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="13" t="n">
         <v>500</v>
       </c>
-      <c r="D15" s="14" t="n">
+      <c r="D15" s="13" t="n">
         <v>140</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="13">
         <f>C15*D15</f>
         <v/>
       </c>
     </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="15" t="n">
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette verte 5,5cm X 5,5cm (année 2028, n°0001 à 1000)</t>
         </is>
       </c>
-      <c r="C16" s="17" t="n">
+      <c r="C16" s="16" t="n">
         <v>1000</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="16" t="n">
         <v>140</v>
       </c>
-      <c r="E16" s="17">
+      <c r="E16" s="16">
         <f>C16*D16</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="12" t="n">
+    <row r="17" ht="17" customHeight="1">
+      <c r="A17" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette orange 5,5cm X 5,5cm (n°2001 à 3000)</t>
         </is>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C17" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="D17" s="14" t="n">
+      <c r="D17" s="13" t="n">
         <v>140</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="13">
         <f>C17*D17</f>
         <v/>
       </c>
     </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="15" t="n">
+    <row r="18" ht="17" customHeight="1">
+      <c r="A18" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette rouge 5,5cm X 5,5cm (n°2001 à 3000)</t>
         </is>
       </c>
-      <c r="C18" s="17" t="n">
+      <c r="C18" s="16" t="n">
         <v>1000</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="16" t="n">
         <v>140</v>
       </c>
-      <c r="E18" s="17">
+      <c r="E18" s="16">
         <f>C18*D18</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="12" t="n">
+    <row r="19" ht="17" customHeight="1">
+      <c r="A19" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B19" s="13" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette verte 5cm X 2cm (année 2027, n°401 à 650)</t>
         </is>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C19" s="13" t="n">
         <v>250</v>
       </c>
-      <c r="D19" s="14" t="n">
+      <c r="D19" s="13" t="n">
         <v>120</v>
       </c>
-      <c r="E19" s="14">
+      <c r="E19" s="13">
         <f>C19*D19</f>
         <v/>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="15" t="n">
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Conception/Impression étiquette verte 5cm X 2cm (année 2028, n°1 à 250)</t>
         </is>
       </c>
-      <c r="C20" s="17" t="n">
+      <c r="C20" s="16" t="n">
         <v>250</v>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="16" t="n">
         <v>120</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E20" s="16">
         <f>C20*D20</f>
         <v/>
       </c>
     </row>
-    <row r="21" ht="22" customHeight="1">
-      <c r="A21" s="12" t="n">
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B21" s="13" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>Scellé de sécurité personnalisés (câble acier &amp; corps polycarbonate inviolable)</t>
         </is>
       </c>
-      <c r="C21" s="14" t="n">
+      <c r="C21" s="13" t="n">
         <v>1000</v>
       </c>
-      <c r="D21" s="14" t="n">
+      <c r="D21" s="13" t="n">
         <v>1370</v>
       </c>
-      <c r="E21" s="14">
+      <c r="E21" s="13">
         <f>C21*D21</f>
         <v/>
       </c>
     </row>
-    <row r="22" ht="25" customHeight="1">
-      <c r="A22" s="18" t="inlineStr">
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>TOTAL GÉNÉRAL HORS TAXES (HT) FCFA</t>
         </is>
       </c>
-      <c r="B22" s="19" t="n"/>
-      <c r="C22" s="19" t="n"/>
-      <c r="D22" s="19" t="n"/>
-      <c r="E22" s="20">
+      <c r="B22" s="18" t="n"/>
+      <c r="C22" s="18" t="n"/>
+      <c r="D22" s="18" t="n"/>
+      <c r="E22" s="19">
         <f>SUM(E11:E21)</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="21" t="inlineStr">
-        <is>
-          <t>Arrêtée la présente facture proforma à la somme de : QUATRE MILLIONS NEUF CENT VINGT MILLE (4 920 000) FRANCS CFA HORS TAXES.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+    <row r="23" ht="6" customHeight="1"/>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="20" t="inlineStr">
+        <is>
+          <t>Arrêtée la présente facture proforma à la somme de : QUATRE MILLIONS NEUF CENT VINGT MILLE (4 920 000) FCFA HT.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="6" customHeight="1"/>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="21" t="inlineStr">
         <is>
           <t>TERMES ET CONDITIONS D'EXÉCUTION :</t>
         </is>
       </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>• Délai de livraison : 35 à 50 jours calendaires après validation définitive du Bon À Tirer (BAT) et signature du marché.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>• Conditions de règlement : 50% d'acompte à la commande, solde à la livraison sur présentation de la facture définitive.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>• Garantie qualité : Matière polyester indéchirable, adhésif renforcé résistant aux solvants, intempéries et écarts thermiques.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>• Domiciliation bancaire : BANK OF AFRICA (BOA NIGER) Niamey | N° Compte: 00125478901-54 | Clé: 18</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>Pour SGSI SA,</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="D33" s="8" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
+        <is>
+          <t>Pour SGSI SA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>• Délai de livraison : 35 à 50 jours calendaires après signature du contrat et approbation du BAT.</t>
+        </is>
+      </c>
+      <c r="D27" s="23" t="inlineStr">
         <is>
           <t>Le Directeur Général</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>[Cachet &amp; Signature Électronique]</t>
+    <row r="28" ht="13" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>• Conditions de règlement : 50% d'acompte à la commande, solde à la livraison sur facture définitive.</t>
+        </is>
+      </c>
+      <c r="D28" s="24" t="inlineStr">
+        <is>
+          <t>[Cachet &amp; Signature]</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="13" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>• Spécifications : Support polyester indéchirable, adhésif renforcé résistant aux solvants et aux UV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="13" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>• Domiciliation : BANK OF AFRICA (BOA NIGER) Niamey | N° Compte: 00125478901-54 | Clé: 18</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="16" customHeight="1">
+      <c r="A31" s="25" t="inlineStr">
+        <is>
+          <t>« SGSI SA — Société Anonyme au capital de 25 000 000 FCFA — Niamey, Niger »</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A29:E29"/>
+  <mergeCells count="20">
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="D1:E1"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="D7:E7"/>
-    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="D28:E30"/>
+    <mergeCell ref="A8:E8"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A6:E6"/>
-    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A31:E31"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A8:E8"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="D26:E26"/>
   </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <printOptions horizontalCentered="1" verticalCentered="0" gridLines="0"/>
+  <pageMargins left="0.35" right="0.35" top="0.35" bottom="0.35" header="0.2" footer="0.2"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>